<commit_message>
Korrekturen in Datenbank und Heat diagramm in FT Modellen
Wärmespeicher Outputs in Excel --> Einheiten korrigiert auf kWh_th
3.2.2.7 Beschriftung in MW, Werte aber eig in kW --> /1000 ergänzt
4.1.3 - Einheit für Wärme wird als t/a angegeben --> GWh/a in eigenes Diagramm
</commit_message>
<xml_diff>
--- a/Fischer_Tropsch/FischerTropsch_Greenfield_Patagonien/Datenbank.xlsx
+++ b/Fischer_Tropsch/FischerTropsch_Greenfield_Patagonien/Datenbank.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01-Arbeit\06-FENES\09-P2X3\FENES_P2X\Fischer_Tropsch\FischerTropsch_Greenfield_Patagonien\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E86C701A-53F8-4A6D-A023-54646A5DF089}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A4835E4-8517-47F6-9951-2D471768D49D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="23520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datenauswahl" sheetId="1" r:id="rId1"/>
@@ -181,7 +181,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="375">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="376">
   <si>
     <t>PEM Elektrolyse</t>
   </si>
@@ -1308,6 +1308,9 @@
   </si>
   <si>
     <t>calc_price</t>
+  </si>
+  <si>
+    <t>kWh_th/a</t>
   </si>
 </sst>
 </file>
@@ -1320,7 +1323,7 @@
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1370,14 +1373,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FFFFC000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color rgb="FFFFC000"/>
       <name val="Calibri"/>
@@ -1530,9 +1525,9 @@
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="107">
+  <cellXfs count="105">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -1588,30 +1583,31 @@
     <xf numFmtId="2" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="2" fontId="14" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="13" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1666,14 +1662,20 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1681,8 +1683,14 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1690,39 +1698,20 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2248,10 +2237,10 @@
       <c r="G1" s="6"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="69" t="s">
+      <c r="A2" s="70" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="79" t="s">
+      <c r="B2" s="80" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
@@ -2268,8 +2257,8 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="70"/>
-      <c r="B3" s="77"/>
+      <c r="A3" s="71"/>
+      <c r="B3" s="78"/>
       <c r="C3" t="s">
         <v>84</v>
       </c>
@@ -2284,8 +2273,8 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="70"/>
-      <c r="B4" s="77"/>
+      <c r="A4" s="71"/>
+      <c r="B4" s="78"/>
       <c r="C4" t="s">
         <v>10</v>
       </c>
@@ -2300,8 +2289,8 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="70"/>
-      <c r="B5" s="77"/>
+      <c r="A5" s="71"/>
+      <c r="B5" s="78"/>
       <c r="C5" t="s">
         <v>11</v>
       </c>
@@ -2316,8 +2305,8 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="70"/>
-      <c r="B6" s="77"/>
+      <c r="A6" s="71"/>
+      <c r="B6" s="78"/>
       <c r="C6" t="s">
         <v>13</v>
       </c>
@@ -2332,8 +2321,8 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="70"/>
-      <c r="B7" s="77"/>
+      <c r="A7" s="71"/>
+      <c r="B7" s="78"/>
       <c r="C7" t="s">
         <v>15</v>
       </c>
@@ -2348,8 +2337,8 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="70"/>
-      <c r="B8" s="80" t="s">
+      <c r="A8" s="71"/>
+      <c r="B8" s="81" t="s">
         <v>332</v>
       </c>
       <c r="C8" s="35" t="s">
@@ -2366,8 +2355,8 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="70"/>
-      <c r="B9" s="81"/>
+      <c r="A9" s="71"/>
+      <c r="B9" s="82"/>
       <c r="C9" s="13" t="s">
         <v>85</v>
       </c>
@@ -2382,8 +2371,8 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="70"/>
-      <c r="B10" s="81"/>
+      <c r="A10" s="71"/>
+      <c r="B10" s="82"/>
       <c r="C10" s="13" t="s">
         <v>10</v>
       </c>
@@ -2398,8 +2387,8 @@
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="70"/>
-      <c r="B11" s="81"/>
+      <c r="A11" s="71"/>
+      <c r="B11" s="82"/>
       <c r="C11" s="13" t="s">
         <v>11</v>
       </c>
@@ -2414,8 +2403,8 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="70"/>
-      <c r="B12" s="81"/>
+      <c r="A12" s="71"/>
+      <c r="B12" s="82"/>
       <c r="C12" s="13" t="s">
         <v>86</v>
       </c>
@@ -2430,8 +2419,8 @@
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="70"/>
-      <c r="B13" s="81"/>
+      <c r="A13" s="71"/>
+      <c r="B13" s="82"/>
       <c r="C13" s="13" t="s">
         <v>239</v>
       </c>
@@ -2446,8 +2435,8 @@
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="70"/>
-      <c r="B14" s="81"/>
+      <c r="A14" s="71"/>
+      <c r="B14" s="82"/>
       <c r="C14" s="13" t="s">
         <v>13</v>
       </c>
@@ -2462,8 +2451,8 @@
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="70"/>
-      <c r="B15" s="82"/>
+      <c r="A15" s="71"/>
+      <c r="B15" s="83"/>
       <c r="C15" s="36" t="s">
         <v>15</v>
       </c>
@@ -2478,8 +2467,8 @@
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="70"/>
-      <c r="B16" s="84" t="s">
+      <c r="A16" s="71"/>
+      <c r="B16" s="85" t="s">
         <v>264</v>
       </c>
       <c r="C16" s="35" t="s">
@@ -2496,8 +2485,8 @@
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="70"/>
-      <c r="B17" s="85"/>
+      <c r="A17" s="71"/>
+      <c r="B17" s="86"/>
       <c r="C17" s="13" t="s">
         <v>84</v>
       </c>
@@ -2512,8 +2501,8 @@
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="70"/>
-      <c r="B18" s="85"/>
+      <c r="A18" s="71"/>
+      <c r="B18" s="86"/>
       <c r="C18" s="13" t="s">
         <v>10</v>
       </c>
@@ -2528,8 +2517,8 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="70"/>
-      <c r="B19" s="85"/>
+      <c r="A19" s="71"/>
+      <c r="B19" s="86"/>
       <c r="C19" s="13" t="s">
         <v>11</v>
       </c>
@@ -2544,8 +2533,8 @@
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="70"/>
-      <c r="B20" s="85"/>
+      <c r="A20" s="71"/>
+      <c r="B20" s="86"/>
       <c r="C20" s="13" t="s">
         <v>13</v>
       </c>
@@ -2560,8 +2549,8 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="70"/>
-      <c r="B21" s="86"/>
+      <c r="A21" s="71"/>
+      <c r="B21" s="87"/>
       <c r="C21" s="36" t="s">
         <v>15</v>
       </c>
@@ -2576,8 +2565,8 @@
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="70"/>
-      <c r="B22" s="83" t="s">
+      <c r="A22" s="71"/>
+      <c r="B22" s="84" t="s">
         <v>231</v>
       </c>
       <c r="C22" s="44" t="s">
@@ -2594,8 +2583,8 @@
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="70"/>
-      <c r="B23" s="83"/>
+      <c r="A23" s="71"/>
+      <c r="B23" s="84"/>
       <c r="C23" s="44" t="s">
         <v>272</v>
       </c>
@@ -2610,8 +2599,8 @@
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="70"/>
-      <c r="B24" s="83"/>
+      <c r="A24" s="71"/>
+      <c r="B24" s="84"/>
       <c r="C24" s="44" t="s">
         <v>10</v>
       </c>
@@ -2626,8 +2615,8 @@
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="70"/>
-      <c r="B25" s="83"/>
+      <c r="A25" s="71"/>
+      <c r="B25" s="84"/>
       <c r="C25" s="44" t="s">
         <v>11</v>
       </c>
@@ -2642,8 +2631,8 @@
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="70"/>
-      <c r="B26" s="83"/>
+      <c r="A26" s="71"/>
+      <c r="B26" s="84"/>
       <c r="C26" s="44" t="s">
         <v>13</v>
       </c>
@@ -2658,8 +2647,8 @@
       </c>
     </row>
     <row r="27" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="70"/>
-      <c r="B27" s="83"/>
+      <c r="A27" s="71"/>
+      <c r="B27" s="84"/>
       <c r="C27" s="44" t="s">
         <v>15</v>
       </c>
@@ -2674,10 +2663,10 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="69" t="s">
+      <c r="A28" s="70" t="s">
         <v>71</v>
       </c>
-      <c r="B28" s="72" t="s">
+      <c r="B28" s="73" t="s">
         <v>3</v>
       </c>
       <c r="C28" s="2" t="s">
@@ -2694,8 +2683,8 @@
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="70"/>
-      <c r="B29" s="73"/>
+      <c r="A29" s="71"/>
+      <c r="B29" s="74"/>
       <c r="C29" t="s">
         <v>11</v>
       </c>
@@ -2710,8 +2699,8 @@
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="70"/>
-      <c r="B30" s="73"/>
+      <c r="A30" s="71"/>
+      <c r="B30" s="74"/>
       <c r="C30" t="s">
         <v>13</v>
       </c>
@@ -2726,8 +2715,8 @@
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="70"/>
-      <c r="B31" s="73"/>
+      <c r="A31" s="71"/>
+      <c r="B31" s="74"/>
       <c r="C31" t="s">
         <v>20</v>
       </c>
@@ -2742,8 +2731,8 @@
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="70"/>
-      <c r="B32" s="73"/>
+      <c r="A32" s="71"/>
+      <c r="B32" s="74"/>
       <c r="C32" t="s">
         <v>35</v>
       </c>
@@ -2758,8 +2747,8 @@
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="70"/>
-      <c r="B33" s="73"/>
+      <c r="A33" s="71"/>
+      <c r="B33" s="74"/>
       <c r="C33" t="s">
         <v>36</v>
       </c>
@@ -2774,8 +2763,8 @@
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="70"/>
-      <c r="B34" s="73"/>
+      <c r="A34" s="71"/>
+      <c r="B34" s="74"/>
       <c r="C34" t="s">
         <v>15</v>
       </c>
@@ -2790,8 +2779,8 @@
       </c>
     </row>
     <row r="35" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="70"/>
-      <c r="B35" s="74"/>
+      <c r="A35" s="71"/>
+      <c r="B35" s="75"/>
       <c r="C35" s="5" t="s">
         <v>88</v>
       </c>
@@ -2806,8 +2795,8 @@
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="70"/>
-      <c r="B36" s="75" t="s">
+      <c r="A36" s="71"/>
+      <c r="B36" s="76" t="s">
         <v>307</v>
       </c>
       <c r="C36" s="26" t="s">
@@ -2824,8 +2813,8 @@
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="70"/>
-      <c r="B37" s="73"/>
+      <c r="A37" s="71"/>
+      <c r="B37" s="74"/>
       <c r="C37" s="13" t="s">
         <v>11</v>
       </c>
@@ -2840,8 +2829,8 @@
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="70"/>
-      <c r="B38" s="73"/>
+      <c r="A38" s="71"/>
+      <c r="B38" s="74"/>
       <c r="C38" s="13" t="s">
         <v>13</v>
       </c>
@@ -2856,8 +2845,8 @@
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="70"/>
-      <c r="B39" s="73"/>
+      <c r="A39" s="71"/>
+      <c r="B39" s="74"/>
       <c r="C39" s="13" t="s">
         <v>20</v>
       </c>
@@ -2872,8 +2861,8 @@
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="70"/>
-      <c r="B40" s="73"/>
+      <c r="A40" s="71"/>
+      <c r="B40" s="74"/>
       <c r="C40" s="13" t="s">
         <v>35</v>
       </c>
@@ -2888,8 +2877,8 @@
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="70"/>
-      <c r="B41" s="73"/>
+      <c r="A41" s="71"/>
+      <c r="B41" s="74"/>
       <c r="C41" s="13" t="s">
         <v>36</v>
       </c>
@@ -2904,8 +2893,8 @@
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="70"/>
-      <c r="B42" s="73"/>
+      <c r="A42" s="71"/>
+      <c r="B42" s="74"/>
       <c r="C42" s="13" t="s">
         <v>15</v>
       </c>
@@ -2920,8 +2909,8 @@
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43" s="70"/>
-      <c r="B43" s="73"/>
+      <c r="A43" s="71"/>
+      <c r="B43" s="74"/>
       <c r="C43" s="36" t="s">
         <v>88</v>
       </c>
@@ -2936,8 +2925,8 @@
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A44" s="70"/>
-      <c r="B44" s="75" t="s">
+      <c r="A44" s="71"/>
+      <c r="B44" s="76" t="s">
         <v>203</v>
       </c>
       <c r="C44" s="4" t="s">
@@ -2954,8 +2943,8 @@
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A45" s="70"/>
-      <c r="B45" s="77"/>
+      <c r="A45" s="71"/>
+      <c r="B45" s="78"/>
       <c r="C45" t="s">
         <v>21</v>
       </c>
@@ -2971,8 +2960,8 @@
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A46" s="70"/>
-      <c r="B46" s="77"/>
+      <c r="A46" s="71"/>
+      <c r="B46" s="78"/>
       <c r="C46" t="s">
         <v>16</v>
       </c>
@@ -2987,8 +2976,8 @@
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47" s="70"/>
-      <c r="B47" s="77"/>
+      <c r="A47" s="71"/>
+      <c r="B47" s="78"/>
       <c r="C47" t="s">
         <v>17</v>
       </c>
@@ -3003,8 +2992,8 @@
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48" s="70"/>
-      <c r="B48" s="77"/>
+      <c r="A48" s="71"/>
+      <c r="B48" s="78"/>
       <c r="C48" t="s">
         <v>35</v>
       </c>
@@ -3019,8 +3008,8 @@
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="70"/>
-      <c r="B49" s="77"/>
+      <c r="A49" s="71"/>
+      <c r="B49" s="78"/>
       <c r="C49" t="s">
         <v>36</v>
       </c>
@@ -3035,8 +3024,8 @@
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A50" s="70"/>
-      <c r="B50" s="77"/>
+      <c r="A50" s="71"/>
+      <c r="B50" s="78"/>
       <c r="C50" t="s">
         <v>89</v>
       </c>
@@ -3051,8 +3040,8 @@
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A51" s="70"/>
-      <c r="B51" s="77"/>
+      <c r="A51" s="71"/>
+      <c r="B51" s="78"/>
       <c r="C51" t="s">
         <v>88</v>
       </c>
@@ -3067,8 +3056,8 @@
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A52" s="70"/>
-      <c r="B52" s="77"/>
+      <c r="A52" s="71"/>
+      <c r="B52" s="78"/>
       <c r="C52" t="s">
         <v>13</v>
       </c>
@@ -3083,8 +3072,8 @@
       </c>
     </row>
     <row r="53" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="71"/>
-      <c r="B53" s="78"/>
+      <c r="A53" s="72"/>
+      <c r="B53" s="79"/>
       <c r="C53" s="15" t="s">
         <v>15</v>
       </c>
@@ -3099,7 +3088,7 @@
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A54" s="69" t="s">
+      <c r="A54" s="70" t="s">
         <v>72</v>
       </c>
       <c r="B54" s="11" t="s">
@@ -3119,8 +3108,8 @@
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A55" s="70"/>
-      <c r="B55" s="75" t="s">
+      <c r="A55" s="71"/>
+      <c r="B55" s="76" t="s">
         <v>4</v>
       </c>
       <c r="C55" s="4" t="s">
@@ -3137,8 +3126,8 @@
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A56" s="70"/>
-      <c r="B56" s="73"/>
+      <c r="A56" s="71"/>
+      <c r="B56" s="74"/>
       <c r="C56" t="s">
         <v>10</v>
       </c>
@@ -3153,8 +3142,8 @@
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" s="70"/>
-      <c r="B57" s="73"/>
+      <c r="A57" s="71"/>
+      <c r="B57" s="74"/>
       <c r="C57" t="s">
         <v>17</v>
       </c>
@@ -3169,8 +3158,8 @@
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" s="70"/>
-      <c r="B58" s="73"/>
+      <c r="A58" s="71"/>
+      <c r="B58" s="74"/>
       <c r="C58" t="s">
         <v>18</v>
       </c>
@@ -3185,8 +3174,8 @@
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A59" s="70"/>
-      <c r="B59" s="73"/>
+      <c r="A59" s="71"/>
+      <c r="B59" s="74"/>
       <c r="C59" t="s">
         <v>13</v>
       </c>
@@ -3201,8 +3190,8 @@
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A60" s="70"/>
-      <c r="B60" s="73"/>
+      <c r="A60" s="71"/>
+      <c r="B60" s="74"/>
       <c r="C60" t="s">
         <v>68</v>
       </c>
@@ -3217,8 +3206,8 @@
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A61" s="70"/>
-      <c r="B61" s="74"/>
+      <c r="A61" s="71"/>
+      <c r="B61" s="75"/>
       <c r="C61" s="5" t="s">
         <v>15</v>
       </c>
@@ -3233,8 +3222,8 @@
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A62" s="70"/>
-      <c r="B62" s="75" t="s">
+      <c r="A62" s="71"/>
+      <c r="B62" s="76" t="s">
         <v>5</v>
       </c>
       <c r="C62" s="4" t="s">
@@ -3251,8 +3240,8 @@
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A63" s="70"/>
-      <c r="B63" s="73"/>
+      <c r="A63" s="71"/>
+      <c r="B63" s="74"/>
       <c r="C63" t="s">
         <v>10</v>
       </c>
@@ -3267,8 +3256,8 @@
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A64" s="70"/>
-      <c r="B64" s="73"/>
+      <c r="A64" s="71"/>
+      <c r="B64" s="74"/>
       <c r="C64" t="s">
         <v>17</v>
       </c>
@@ -3283,8 +3272,8 @@
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A65" s="70"/>
-      <c r="B65" s="73"/>
+      <c r="A65" s="71"/>
+      <c r="B65" s="74"/>
       <c r="C65" t="s">
         <v>18</v>
       </c>
@@ -3299,8 +3288,8 @@
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A66" s="70"/>
-      <c r="B66" s="73"/>
+      <c r="A66" s="71"/>
+      <c r="B66" s="74"/>
       <c r="C66" t="s">
         <v>13</v>
       </c>
@@ -3315,8 +3304,8 @@
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A67" s="70"/>
-      <c r="B67" s="73"/>
+      <c r="A67" s="71"/>
+      <c r="B67" s="74"/>
       <c r="C67" t="s">
         <v>68</v>
       </c>
@@ -3331,8 +3320,8 @@
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A68" s="71"/>
-      <c r="B68" s="76"/>
+      <c r="A68" s="72"/>
+      <c r="B68" s="77"/>
       <c r="C68" s="15" t="s">
         <v>15</v>
       </c>
@@ -3347,7 +3336,7 @@
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A69" s="69" t="s">
+      <c r="A69" s="70" t="s">
         <v>76</v>
       </c>
       <c r="B69" s="56" t="s">
@@ -3367,7 +3356,7 @@
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A70" s="70"/>
+      <c r="A70" s="71"/>
       <c r="B70" s="6" t="s">
         <v>290</v>
       </c>
@@ -3381,11 +3370,11 @@
         <v>-1E-4</v>
       </c>
       <c r="F70" t="s">
-        <v>19</v>
+        <v>316</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A71" s="70"/>
+      <c r="A71" s="71"/>
       <c r="B71" s="17" t="s">
         <v>79</v>
       </c>
@@ -3403,7 +3392,7 @@
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A72" s="71"/>
+      <c r="A72" s="72"/>
       <c r="B72" s="61" t="s">
         <v>333</v>
       </c>
@@ -3477,10 +3466,10 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="87" t="s">
+      <c r="A2" s="91" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="89" t="s">
+      <c r="B2" s="96" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="26" t="s">
@@ -3495,8 +3484,8 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="88"/>
-      <c r="B3" s="85"/>
+      <c r="A3" s="97"/>
+      <c r="B3" s="86"/>
       <c r="C3" s="13" t="s">
         <v>108</v>
       </c>
@@ -3509,8 +3498,8 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="88"/>
-      <c r="B4" s="85"/>
+      <c r="A4" s="97"/>
+      <c r="B4" s="86"/>
       <c r="C4" s="13" t="s">
         <v>84</v>
       </c>
@@ -3523,8 +3512,8 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="88"/>
-      <c r="B5" s="85"/>
+      <c r="A5" s="97"/>
+      <c r="B5" s="86"/>
       <c r="C5" s="13" t="s">
         <v>139</v>
       </c>
@@ -3537,8 +3526,8 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="88"/>
-      <c r="B6" s="85"/>
+      <c r="A6" s="97"/>
+      <c r="B6" s="86"/>
       <c r="C6" s="13" t="s">
         <v>142</v>
       </c>
@@ -3551,8 +3540,8 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="88"/>
-      <c r="B7" s="85"/>
+      <c r="A7" s="97"/>
+      <c r="B7" s="86"/>
       <c r="C7" s="13" t="s">
         <v>156</v>
       </c>
@@ -3565,8 +3554,8 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="88"/>
-      <c r="B8" s="85"/>
+      <c r="A8" s="97"/>
+      <c r="B8" s="86"/>
       <c r="C8" s="13" t="s">
         <v>198</v>
       </c>
@@ -3579,8 +3568,8 @@
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="88"/>
-      <c r="B9" s="85"/>
+      <c r="A9" s="97"/>
+      <c r="B9" s="86"/>
       <c r="C9" s="13" t="s">
         <v>168</v>
       </c>
@@ -3593,8 +3582,8 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="88"/>
-      <c r="B10" s="85"/>
+      <c r="A10" s="97"/>
+      <c r="B10" s="86"/>
       <c r="C10" s="13" t="s">
         <v>190</v>
       </c>
@@ -3607,13 +3596,13 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="88"/>
-      <c r="B11" s="85"/>
+      <c r="A11" s="97"/>
+      <c r="B11" s="86"/>
       <c r="E11" s="33"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="88"/>
-      <c r="B12" s="90" t="s">
+      <c r="A12" s="97"/>
+      <c r="B12" s="93" t="s">
         <v>366</v>
       </c>
       <c r="C12" s="35" t="s">
@@ -3628,8 +3617,8 @@
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="88"/>
-      <c r="B13" s="91"/>
+      <c r="A13" s="97"/>
+      <c r="B13" s="94"/>
       <c r="C13" s="13" t="s">
         <v>365</v>
       </c>
@@ -3642,8 +3631,8 @@
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="88"/>
-      <c r="B14" s="91"/>
+      <c r="A14" s="97"/>
+      <c r="B14" s="94"/>
       <c r="C14" s="13" t="s">
         <v>140</v>
       </c>
@@ -3656,8 +3645,8 @@
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="88"/>
-      <c r="B15" s="91"/>
+      <c r="A15" s="97"/>
+      <c r="B15" s="94"/>
       <c r="C15" s="13" t="s">
         <v>240</v>
       </c>
@@ -3670,8 +3659,8 @@
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="88"/>
-      <c r="B16" s="91"/>
+      <c r="A16" s="97"/>
+      <c r="B16" s="94"/>
       <c r="C16" s="13" t="s">
         <v>84</v>
       </c>
@@ -3684,8 +3673,8 @@
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="88"/>
-      <c r="B17" s="91"/>
+      <c r="A17" s="97"/>
+      <c r="B17" s="94"/>
       <c r="C17" s="13" t="s">
         <v>142</v>
       </c>
@@ -3698,8 +3687,8 @@
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="88"/>
-      <c r="B18" s="91"/>
+      <c r="A18" s="97"/>
+      <c r="B18" s="94"/>
       <c r="C18" s="13" t="s">
         <v>156</v>
       </c>
@@ -3712,8 +3701,8 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="88"/>
-      <c r="B19" s="91"/>
+      <c r="A19" s="97"/>
+      <c r="B19" s="94"/>
       <c r="C19" s="13" t="s">
         <v>198</v>
       </c>
@@ -3726,8 +3715,8 @@
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="88"/>
-      <c r="B20" s="91"/>
+      <c r="A20" s="97"/>
+      <c r="B20" s="94"/>
       <c r="C20" s="13" t="s">
         <v>168</v>
       </c>
@@ -3740,8 +3729,8 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="88"/>
-      <c r="B21" s="91"/>
+      <c r="A21" s="97"/>
+      <c r="B21" s="94"/>
       <c r="C21" s="13" t="s">
         <v>190</v>
       </c>
@@ -3754,16 +3743,16 @@
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="88"/>
-      <c r="B22" s="92"/>
+      <c r="A22" s="97"/>
+      <c r="B22" s="102"/>
       <c r="C22" s="36"/>
       <c r="D22" s="36"/>
       <c r="E22" s="37"/>
       <c r="F22" s="36"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="88"/>
-      <c r="B23" s="84" t="s">
+      <c r="A23" s="97"/>
+      <c r="B23" s="85" t="s">
         <v>264</v>
       </c>
       <c r="C23" s="13" t="s">
@@ -3778,8 +3767,8 @@
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="88"/>
-      <c r="B24" s="85"/>
+      <c r="A24" s="97"/>
+      <c r="B24" s="86"/>
       <c r="C24" s="13" t="s">
         <v>108</v>
       </c>
@@ -3792,8 +3781,8 @@
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="88"/>
-      <c r="B25" s="85"/>
+      <c r="A25" s="97"/>
+      <c r="B25" s="86"/>
       <c r="C25" s="13" t="s">
         <v>84</v>
       </c>
@@ -3806,8 +3795,8 @@
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="88"/>
-      <c r="B26" s="85"/>
+      <c r="A26" s="97"/>
+      <c r="B26" s="86"/>
       <c r="C26" s="13" t="s">
         <v>285</v>
       </c>
@@ -3820,8 +3809,8 @@
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="88"/>
-      <c r="B27" s="85"/>
+      <c r="A27" s="97"/>
+      <c r="B27" s="86"/>
       <c r="C27" s="13" t="s">
         <v>142</v>
       </c>
@@ -3834,8 +3823,8 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="88"/>
-      <c r="B28" s="85"/>
+      <c r="A28" s="97"/>
+      <c r="B28" s="86"/>
       <c r="C28" s="13" t="s">
         <v>156</v>
       </c>
@@ -3848,8 +3837,8 @@
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="88"/>
-      <c r="B29" s="85"/>
+      <c r="A29" s="97"/>
+      <c r="B29" s="86"/>
       <c r="C29" s="13" t="s">
         <v>198</v>
       </c>
@@ -3862,8 +3851,8 @@
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="88"/>
-      <c r="B30" s="85"/>
+      <c r="A30" s="97"/>
+      <c r="B30" s="86"/>
       <c r="C30" s="13" t="s">
         <v>168</v>
       </c>
@@ -3876,8 +3865,8 @@
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="88"/>
-      <c r="B31" s="85"/>
+      <c r="A31" s="97"/>
+      <c r="B31" s="86"/>
       <c r="C31" s="13" t="s">
         <v>190</v>
       </c>
@@ -3890,16 +3879,16 @@
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="88"/>
-      <c r="B32" s="86"/>
+      <c r="A32" s="97"/>
+      <c r="B32" s="87"/>
       <c r="C32" s="36"/>
       <c r="D32" s="36"/>
       <c r="E32" s="37"/>
       <c r="F32" s="36"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="88"/>
-      <c r="B33" s="83" t="s">
+      <c r="A33" s="97"/>
+      <c r="B33" s="84" t="s">
         <v>231</v>
       </c>
       <c r="C33" s="13" t="s">
@@ -3914,8 +3903,8 @@
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="88"/>
-      <c r="B34" s="83"/>
+      <c r="A34" s="97"/>
+      <c r="B34" s="84"/>
       <c r="C34" s="13" t="s">
         <v>108</v>
       </c>
@@ -3928,8 +3917,8 @@
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="88"/>
-      <c r="B35" s="83"/>
+      <c r="A35" s="97"/>
+      <c r="B35" s="84"/>
       <c r="C35" s="13" t="s">
         <v>84</v>
       </c>
@@ -3942,8 +3931,8 @@
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="88"/>
-      <c r="B36" s="83"/>
+      <c r="A36" s="97"/>
+      <c r="B36" s="84"/>
       <c r="C36" s="13" t="s">
         <v>272</v>
       </c>
@@ -3956,8 +3945,8 @@
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="88"/>
-      <c r="B37" s="83"/>
+      <c r="A37" s="97"/>
+      <c r="B37" s="84"/>
       <c r="C37" s="13" t="s">
         <v>250</v>
       </c>
@@ -3970,8 +3959,8 @@
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="88"/>
-      <c r="B38" s="83"/>
+      <c r="A38" s="97"/>
+      <c r="B38" s="84"/>
       <c r="C38" s="13" t="s">
         <v>142</v>
       </c>
@@ -3984,8 +3973,8 @@
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="88"/>
-      <c r="B39" s="83"/>
+      <c r="A39" s="97"/>
+      <c r="B39" s="84"/>
       <c r="C39" s="13" t="s">
         <v>156</v>
       </c>
@@ -3998,8 +3987,8 @@
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="88"/>
-      <c r="B40" s="83"/>
+      <c r="A40" s="97"/>
+      <c r="B40" s="84"/>
       <c r="C40" s="13" t="s">
         <v>198</v>
       </c>
@@ -4012,8 +4001,8 @@
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="88"/>
-      <c r="B41" s="83"/>
+      <c r="A41" s="97"/>
+      <c r="B41" s="84"/>
       <c r="C41" s="13" t="s">
         <v>168</v>
       </c>
@@ -4026,8 +4015,8 @@
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="88"/>
-      <c r="B42" s="83"/>
+      <c r="A42" s="97"/>
+      <c r="B42" s="84"/>
       <c r="C42" s="13" t="s">
         <v>190</v>
       </c>
@@ -4040,15 +4029,15 @@
       </c>
     </row>
     <row r="43" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="88"/>
-      <c r="B43" s="83"/>
+      <c r="A43" s="97"/>
+      <c r="B43" s="84"/>
       <c r="E43" s="33"/>
     </row>
     <row r="44" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="87" t="s">
+      <c r="A44" s="91" t="s">
         <v>71</v>
       </c>
-      <c r="B44" s="96" t="s">
+      <c r="B44" s="104" t="s">
         <v>3</v>
       </c>
       <c r="C44" s="26" t="s">
@@ -4063,8 +4052,8 @@
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A45" s="88"/>
-      <c r="B45" s="83"/>
+      <c r="A45" s="97"/>
+      <c r="B45" s="84"/>
       <c r="C45" s="13" t="s">
         <v>112</v>
       </c>
@@ -4077,8 +4066,8 @@
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A46" s="88"/>
-      <c r="B46" s="83"/>
+      <c r="A46" s="97"/>
+      <c r="B46" s="84"/>
       <c r="C46" s="13" t="s">
         <v>136</v>
       </c>
@@ -4091,8 +4080,8 @@
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47" s="88"/>
-      <c r="B47" s="83"/>
+      <c r="A47" s="97"/>
+      <c r="B47" s="84"/>
       <c r="C47" s="13" t="s">
         <v>137</v>
       </c>
@@ -4105,8 +4094,8 @@
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48" s="88"/>
-      <c r="B48" s="83"/>
+      <c r="A48" s="97"/>
+      <c r="B48" s="84"/>
       <c r="C48" s="13" t="s">
         <v>142</v>
       </c>
@@ -4119,8 +4108,8 @@
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="88"/>
-      <c r="B49" s="83"/>
+      <c r="A49" s="97"/>
+      <c r="B49" s="84"/>
       <c r="C49" s="13" t="s">
         <v>156</v>
       </c>
@@ -4133,8 +4122,8 @@
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A50" s="88"/>
-      <c r="B50" s="83"/>
+      <c r="A50" s="97"/>
+      <c r="B50" s="84"/>
       <c r="C50" s="13" t="s">
         <v>198</v>
       </c>
@@ -4147,8 +4136,8 @@
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A51" s="88"/>
-      <c r="B51" s="83"/>
+      <c r="A51" s="97"/>
+      <c r="B51" s="84"/>
       <c r="C51" s="13" t="s">
         <v>168</v>
       </c>
@@ -4161,8 +4150,8 @@
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A52" s="88"/>
-      <c r="B52" s="83"/>
+      <c r="A52" s="97"/>
+      <c r="B52" s="84"/>
       <c r="C52" s="13" t="s">
         <v>190</v>
       </c>
@@ -4175,152 +4164,149 @@
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A53" s="88"/>
-      <c r="B53" s="97"/>
+      <c r="A53" s="97"/>
+      <c r="B53" s="100"/>
       <c r="C53" s="36"/>
       <c r="D53" s="36"/>
       <c r="E53" s="37"/>
       <c r="F53" s="36"/>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A54" s="88"/>
-      <c r="B54" s="98" t="s">
+      <c r="A54" s="97"/>
+      <c r="B54" s="84" t="s">
         <v>307</v>
       </c>
-      <c r="C54" s="44" t="s">
+      <c r="C54" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="D54" s="44" t="s">
+      <c r="D54" s="13" t="s">
         <v>317</v>
       </c>
-      <c r="E54" s="46"/>
-      <c r="F54" s="44" t="s">
+      <c r="E54" s="31"/>
+      <c r="F54" s="13" t="s">
         <v>330</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A55" s="88"/>
-      <c r="B55" s="98"/>
-      <c r="C55" s="44" t="s">
+      <c r="A55" s="97"/>
+      <c r="B55" s="84"/>
+      <c r="C55" s="13" t="s">
         <v>112</v>
       </c>
-      <c r="D55" s="44" t="s">
+      <c r="D55" s="13" t="s">
         <v>318</v>
       </c>
-      <c r="E55" s="47"/>
-      <c r="F55" s="44" t="s">
+      <c r="E55" s="33"/>
+      <c r="F55" s="13" t="s">
         <v>331</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A56" s="88"/>
-      <c r="B56" s="98"/>
-      <c r="C56" s="44" t="s">
+      <c r="A56" s="97"/>
+      <c r="B56" s="84"/>
+      <c r="C56" s="13" t="s">
         <v>136</v>
       </c>
-      <c r="D56" s="44" t="s">
+      <c r="D56" s="13" t="s">
         <v>319</v>
       </c>
-      <c r="E56" s="48"/>
-      <c r="F56" s="59" t="s">
-        <v>133</v>
+      <c r="E56" s="34"/>
+      <c r="F56" s="13" t="s">
+        <v>375</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" s="88"/>
-      <c r="B57" s="98"/>
-      <c r="C57" s="44" t="s">
+      <c r="A57" s="97"/>
+      <c r="B57" s="84"/>
+      <c r="C57" s="13" t="s">
         <v>137</v>
       </c>
-      <c r="D57" s="44" t="s">
+      <c r="D57" s="13" t="s">
         <v>320</v>
       </c>
-      <c r="E57" s="47"/>
-      <c r="F57" s="59" t="s">
-        <v>133</v>
+      <c r="E57" s="33"/>
+      <c r="F57" s="13" t="s">
+        <v>375</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" s="88"/>
-      <c r="B58" s="98"/>
-      <c r="C58" s="44" t="s">
+      <c r="A58" s="97"/>
+      <c r="B58" s="84"/>
+      <c r="C58" s="13" t="s">
         <v>142</v>
       </c>
-      <c r="D58" s="44" t="s">
+      <c r="D58" s="13" t="s">
         <v>321</v>
       </c>
-      <c r="E58" s="47"/>
-      <c r="F58" s="59" t="s">
+      <c r="E58" s="33"/>
+      <c r="F58" s="13" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A59" s="88"/>
-      <c r="B59" s="98"/>
-      <c r="C59" s="44" t="s">
+      <c r="A59" s="97"/>
+      <c r="B59" s="84"/>
+      <c r="C59" s="13" t="s">
         <v>156</v>
       </c>
-      <c r="D59" s="44" t="s">
+      <c r="D59" s="13" t="s">
         <v>322</v>
       </c>
-      <c r="E59" s="47"/>
-      <c r="F59" s="59" t="s">
+      <c r="E59" s="33"/>
+      <c r="F59" s="13" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A60" s="88"/>
-      <c r="B60" s="98"/>
-      <c r="C60" s="44" t="s">
+      <c r="A60" s="97"/>
+      <c r="B60" s="84"/>
+      <c r="C60" s="13" t="s">
         <v>198</v>
       </c>
-      <c r="D60" s="44" t="s">
+      <c r="D60" s="13" t="s">
         <v>323</v>
       </c>
-      <c r="E60" s="47"/>
-      <c r="F60" s="59" t="s">
+      <c r="E60" s="33"/>
+      <c r="F60" s="13" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A61" s="88"/>
-      <c r="B61" s="98"/>
-      <c r="C61" s="44" t="s">
+      <c r="A61" s="97"/>
+      <c r="B61" s="84"/>
+      <c r="C61" s="13" t="s">
         <v>168</v>
       </c>
-      <c r="D61" s="44" t="s">
+      <c r="D61" s="13" t="s">
         <v>324</v>
       </c>
-      <c r="E61" s="47"/>
-      <c r="F61" s="59" t="s">
+      <c r="E61" s="33"/>
+      <c r="F61" s="13" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A62" s="88"/>
-      <c r="B62" s="98"/>
-      <c r="C62" s="44" t="s">
+      <c r="A62" s="97"/>
+      <c r="B62" s="84"/>
+      <c r="C62" s="13" t="s">
         <v>190</v>
       </c>
-      <c r="D62" s="44" t="s">
+      <c r="D62" s="13" t="s">
         <v>325</v>
       </c>
-      <c r="E62" s="47"/>
-      <c r="F62" s="59" t="s">
+      <c r="E62" s="33"/>
+      <c r="F62" s="13" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A63" s="88"/>
-      <c r="B63" s="99"/>
-      <c r="C63" s="44"/>
-      <c r="D63" s="44"/>
-      <c r="E63" s="47"/>
-      <c r="F63" s="44"/>
+      <c r="A63" s="97"/>
+      <c r="B63" s="100"/>
+      <c r="E63" s="33"/>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A64" s="88"/>
-      <c r="B64" s="94" t="s">
+      <c r="A64" s="97"/>
+      <c r="B64" s="99" t="s">
         <v>6</v>
       </c>
       <c r="C64" s="35" t="s">
@@ -4335,8 +4321,8 @@
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A65" s="88"/>
-      <c r="B65" s="83"/>
+      <c r="A65" s="97"/>
+      <c r="B65" s="84"/>
       <c r="C65" s="13" t="s">
         <v>114</v>
       </c>
@@ -4349,8 +4335,8 @@
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A66" s="88"/>
-      <c r="B66" s="85"/>
+      <c r="A66" s="97"/>
+      <c r="B66" s="86"/>
       <c r="C66" s="13" t="s">
         <v>112</v>
       </c>
@@ -4363,8 +4349,8 @@
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A67" s="88"/>
-      <c r="B67" s="85"/>
+      <c r="A67" s="97"/>
+      <c r="B67" s="86"/>
       <c r="C67" s="13" t="s">
         <v>108</v>
       </c>
@@ -4377,8 +4363,8 @@
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A68" s="88"/>
-      <c r="B68" s="85"/>
+      <c r="A68" s="97"/>
+      <c r="B68" s="86"/>
       <c r="C68" s="13" t="s">
         <v>127</v>
       </c>
@@ -4391,8 +4377,8 @@
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A69" s="88"/>
-      <c r="B69" s="85"/>
+      <c r="A69" s="97"/>
+      <c r="B69" s="86"/>
       <c r="C69" s="13" t="s">
         <v>128</v>
       </c>
@@ -4405,8 +4391,8 @@
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A70" s="88"/>
-      <c r="B70" s="85"/>
+      <c r="A70" s="97"/>
+      <c r="B70" s="86"/>
       <c r="C70" s="13" t="s">
         <v>142</v>
       </c>
@@ -4419,8 +4405,8 @@
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A71" s="88"/>
-      <c r="B71" s="85"/>
+      <c r="A71" s="97"/>
+      <c r="B71" s="86"/>
       <c r="C71" s="13" t="s">
         <v>156</v>
       </c>
@@ -4433,8 +4419,8 @@
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A72" s="88"/>
-      <c r="B72" s="85"/>
+      <c r="A72" s="97"/>
+      <c r="B72" s="86"/>
       <c r="C72" s="13" t="s">
         <v>198</v>
       </c>
@@ -4447,8 +4433,8 @@
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A73" s="88"/>
-      <c r="B73" s="85"/>
+      <c r="A73" s="97"/>
+      <c r="B73" s="86"/>
       <c r="C73" s="13" t="s">
         <v>168</v>
       </c>
@@ -4461,8 +4447,8 @@
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A74" s="88"/>
-      <c r="B74" s="85"/>
+      <c r="A74" s="97"/>
+      <c r="B74" s="86"/>
       <c r="C74" s="13" t="s">
         <v>190</v>
       </c>
@@ -4475,18 +4461,18 @@
       </c>
     </row>
     <row r="75" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A75" s="93"/>
-      <c r="B75" s="95"/>
+      <c r="A75" s="98"/>
+      <c r="B75" s="103"/>
       <c r="C75" s="40"/>
       <c r="D75" s="40"/>
       <c r="E75" s="41"/>
       <c r="F75" s="40"/>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A76" s="87" t="s">
+      <c r="A76" s="91" t="s">
         <v>72</v>
       </c>
-      <c r="B76" s="89" t="s">
+      <c r="B76" s="96" t="s">
         <v>73</v>
       </c>
       <c r="C76" s="26" t="s">
@@ -4501,8 +4487,8 @@
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A77" s="88"/>
-      <c r="B77" s="85"/>
+      <c r="A77" s="97"/>
+      <c r="B77" s="86"/>
       <c r="C77" s="13" t="s">
         <v>154</v>
       </c>
@@ -4515,13 +4501,13 @@
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A78" s="88"/>
-      <c r="B78" s="86"/>
+      <c r="A78" s="97"/>
+      <c r="B78" s="87"/>
       <c r="E78" s="31"/>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A79" s="88"/>
-      <c r="B79" s="94" t="s">
+      <c r="A79" s="97"/>
+      <c r="B79" s="99" t="s">
         <v>4</v>
       </c>
       <c r="C79" s="35" t="s">
@@ -4536,8 +4522,8 @@
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A80" s="88"/>
-      <c r="B80" s="83"/>
+      <c r="A80" s="97"/>
+      <c r="B80" s="84"/>
       <c r="C80" s="13" t="s">
         <v>108</v>
       </c>
@@ -4550,8 +4536,8 @@
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A81" s="88"/>
-      <c r="B81" s="83"/>
+      <c r="A81" s="97"/>
+      <c r="B81" s="84"/>
       <c r="C81" s="13" t="s">
         <v>123</v>
       </c>
@@ -4564,8 +4550,8 @@
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A82" s="88"/>
-      <c r="B82" s="83"/>
+      <c r="A82" s="97"/>
+      <c r="B82" s="84"/>
       <c r="C82" s="13" t="s">
         <v>142</v>
       </c>
@@ -4578,8 +4564,8 @@
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A83" s="88"/>
-      <c r="B83" s="83"/>
+      <c r="A83" s="97"/>
+      <c r="B83" s="84"/>
       <c r="C83" s="13" t="s">
         <v>156</v>
       </c>
@@ -4592,8 +4578,8 @@
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A84" s="88"/>
-      <c r="B84" s="83"/>
+      <c r="A84" s="97"/>
+      <c r="B84" s="84"/>
       <c r="C84" s="13" t="s">
         <v>162</v>
       </c>
@@ -4606,8 +4592,8 @@
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A85" s="88"/>
-      <c r="B85" s="83"/>
+      <c r="A85" s="97"/>
+      <c r="B85" s="84"/>
       <c r="C85" s="13" t="s">
         <v>198</v>
       </c>
@@ -4620,8 +4606,8 @@
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A86" s="88"/>
-      <c r="B86" s="83"/>
+      <c r="A86" s="97"/>
+      <c r="B86" s="84"/>
       <c r="C86" s="13" t="s">
         <v>168</v>
       </c>
@@ -4634,8 +4620,8 @@
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A87" s="88"/>
-      <c r="B87" s="83"/>
+      <c r="A87" s="97"/>
+      <c r="B87" s="84"/>
       <c r="C87" s="13" t="s">
         <v>190</v>
       </c>
@@ -4648,12 +4634,12 @@
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A88" s="88"/>
-      <c r="B88" s="97"/>
+      <c r="A88" s="97"/>
+      <c r="B88" s="100"/>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A89" s="88"/>
-      <c r="B89" s="94" t="s">
+      <c r="A89" s="97"/>
+      <c r="B89" s="99" t="s">
         <v>5</v>
       </c>
       <c r="C89" s="35" t="s">
@@ -4668,8 +4654,8 @@
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A90" s="88"/>
-      <c r="B90" s="83"/>
+      <c r="A90" s="97"/>
+      <c r="B90" s="84"/>
       <c r="C90" s="13" t="s">
         <v>109</v>
       </c>
@@ -4682,8 +4668,8 @@
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A91" s="88"/>
-      <c r="B91" s="83"/>
+      <c r="A91" s="97"/>
+      <c r="B91" s="84"/>
       <c r="C91" s="13" t="s">
         <v>121</v>
       </c>
@@ -4696,8 +4682,8 @@
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A92" s="88"/>
-      <c r="B92" s="83"/>
+      <c r="A92" s="97"/>
+      <c r="B92" s="84"/>
       <c r="C92" s="13" t="s">
         <v>142</v>
       </c>
@@ -4710,8 +4696,8 @@
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A93" s="88"/>
-      <c r="B93" s="83"/>
+      <c r="A93" s="97"/>
+      <c r="B93" s="84"/>
       <c r="C93" s="13" t="s">
         <v>156</v>
       </c>
@@ -4724,8 +4710,8 @@
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A94" s="88"/>
-      <c r="B94" s="83"/>
+      <c r="A94" s="97"/>
+      <c r="B94" s="84"/>
       <c r="C94" s="13" t="s">
         <v>162</v>
       </c>
@@ -4738,8 +4724,8 @@
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A95" s="88"/>
-      <c r="B95" s="83"/>
+      <c r="A95" s="97"/>
+      <c r="B95" s="84"/>
       <c r="C95" s="13" t="s">
         <v>198</v>
       </c>
@@ -4752,8 +4738,8 @@
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A96" s="88"/>
-      <c r="B96" s="83"/>
+      <c r="A96" s="97"/>
+      <c r="B96" s="84"/>
       <c r="C96" s="13" t="s">
         <v>168</v>
       </c>
@@ -4766,8 +4752,8 @@
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A97" s="88"/>
-      <c r="B97" s="83"/>
+      <c r="A97" s="97"/>
+      <c r="B97" s="84"/>
       <c r="C97" s="13" t="s">
         <v>190</v>
       </c>
@@ -4780,14 +4766,14 @@
       </c>
     </row>
     <row r="98" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A98" s="93"/>
+      <c r="A98" s="98"/>
       <c r="B98" s="101"/>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A99" s="87" t="s">
+      <c r="A99" s="91" t="s">
         <v>76</v>
       </c>
-      <c r="B99" s="89" t="s">
+      <c r="B99" s="96" t="s">
         <v>73</v>
       </c>
       <c r="C99" s="26" t="s">
@@ -4802,8 +4788,8 @@
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A100" s="88"/>
-      <c r="B100" s="85"/>
+      <c r="A100" s="97"/>
+      <c r="B100" s="86"/>
       <c r="C100" s="13" t="s">
         <v>230</v>
       </c>
@@ -4816,8 +4802,8 @@
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A101" s="88"/>
-      <c r="B101" s="85"/>
+      <c r="A101" s="97"/>
+      <c r="B101" s="86"/>
       <c r="C101" s="13" t="s">
         <v>151</v>
       </c>
@@ -4830,16 +4816,16 @@
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A102" s="88"/>
-      <c r="B102" s="86"/>
+      <c r="A102" s="97"/>
+      <c r="B102" s="87"/>
       <c r="C102" s="36"/>
       <c r="D102" s="36"/>
       <c r="E102" s="37"/>
       <c r="F102" s="36"/>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A103" s="88"/>
-      <c r="B103" s="84" t="s">
+      <c r="A103" s="97"/>
+      <c r="B103" s="85" t="s">
         <v>294</v>
       </c>
       <c r="C103" s="13" t="s">
@@ -4854,8 +4840,8 @@
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A104" s="88"/>
-      <c r="B104" s="85"/>
+      <c r="A104" s="97"/>
+      <c r="B104" s="86"/>
       <c r="C104" s="13" t="s">
         <v>299</v>
       </c>
@@ -4868,8 +4854,8 @@
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A105" s="88"/>
-      <c r="B105" s="85"/>
+      <c r="A105" s="97"/>
+      <c r="B105" s="86"/>
       <c r="C105" s="13" t="s">
         <v>300</v>
       </c>
@@ -4882,13 +4868,13 @@
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A106" s="88"/>
-      <c r="B106" s="86"/>
+      <c r="A106" s="97"/>
+      <c r="B106" s="87"/>
       <c r="E106" s="33"/>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A107" s="88"/>
-      <c r="B107" s="84" t="s">
+      <c r="A107" s="97"/>
+      <c r="B107" s="85" t="s">
         <v>79</v>
       </c>
       <c r="C107" s="35" t="s">
@@ -4903,8 +4889,8 @@
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A108" s="88"/>
-      <c r="B108" s="85"/>
+      <c r="A108" s="97"/>
+      <c r="B108" s="86"/>
       <c r="C108" s="13" t="s">
         <v>152</v>
       </c>
@@ -4917,16 +4903,16 @@
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A109" s="88"/>
-      <c r="B109" s="86"/>
+      <c r="A109" s="97"/>
+      <c r="B109" s="87"/>
       <c r="C109" s="36"/>
       <c r="D109" s="36"/>
       <c r="E109" s="37"/>
       <c r="F109" s="36"/>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A110" s="88"/>
-      <c r="B110" s="90" t="s">
+      <c r="A110" s="97"/>
+      <c r="B110" s="93" t="s">
         <v>333</v>
       </c>
       <c r="C110" s="13" t="s">
@@ -4941,8 +4927,8 @@
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A111" s="88"/>
-      <c r="B111" s="91"/>
+      <c r="A111" s="97"/>
+      <c r="B111" s="94"/>
       <c r="C111" s="13" t="s">
         <v>364</v>
       </c>
@@ -4955,18 +4941,18 @@
       </c>
     </row>
     <row r="112" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A112" s="93"/>
-      <c r="B112" s="100"/>
+      <c r="A112" s="98"/>
+      <c r="B112" s="95"/>
       <c r="C112" s="40"/>
       <c r="D112" s="40"/>
       <c r="E112" s="41"/>
       <c r="F112" s="40"/>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A113" s="87" t="s">
+      <c r="A113" s="91" t="s">
         <v>164</v>
       </c>
-      <c r="B113" s="89" t="s">
+      <c r="B113" s="96" t="s">
         <v>13</v>
       </c>
       <c r="C113" s="26" t="s">
@@ -4981,8 +4967,8 @@
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A114" s="106"/>
-      <c r="B114" s="85"/>
+      <c r="A114" s="92"/>
+      <c r="B114" s="86"/>
       <c r="C114" s="13" t="s">
         <v>175</v>
       </c>
@@ -4994,16 +4980,16 @@
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A115" s="106"/>
-      <c r="B115" s="86"/>
+      <c r="A115" s="92"/>
+      <c r="B115" s="87"/>
       <c r="C115" s="36"/>
       <c r="D115" s="36"/>
       <c r="E115" s="36"/>
       <c r="F115" s="36"/>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A116" s="106"/>
-      <c r="B116" s="84" t="s">
+      <c r="A116" s="92"/>
+      <c r="B116" s="85" t="s">
         <v>184</v>
       </c>
       <c r="C116" s="13" t="s">
@@ -5017,8 +5003,8 @@
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A117" s="106"/>
-      <c r="B117" s="85"/>
+      <c r="A117" s="92"/>
+      <c r="B117" s="86"/>
       <c r="C117" s="13" t="s">
         <v>182</v>
       </c>
@@ -5030,8 +5016,8 @@
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A118" s="106"/>
-      <c r="B118" s="85"/>
+      <c r="A118" s="92"/>
+      <c r="B118" s="86"/>
       <c r="C118" s="13" t="s">
         <v>178</v>
       </c>
@@ -5043,8 +5029,8 @@
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A119" s="106"/>
-      <c r="B119" s="85"/>
+      <c r="A119" s="92"/>
+      <c r="B119" s="86"/>
       <c r="C119" s="13" t="s">
         <v>180</v>
       </c>
@@ -5056,8 +5042,8 @@
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A120" s="106"/>
-      <c r="B120" s="85"/>
+      <c r="A120" s="92"/>
+      <c r="B120" s="86"/>
       <c r="C120" s="13" t="s">
         <v>183</v>
       </c>
@@ -5069,8 +5055,8 @@
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A121" s="106"/>
-      <c r="B121" s="85"/>
+      <c r="A121" s="92"/>
+      <c r="B121" s="86"/>
       <c r="C121" s="13" t="s">
         <v>193</v>
       </c>
@@ -5082,12 +5068,12 @@
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A122" s="106"/>
-      <c r="B122" s="85"/>
+      <c r="A122" s="92"/>
+      <c r="B122" s="86"/>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A123" s="106"/>
-      <c r="B123" s="84" t="s">
+      <c r="A123" s="92"/>
+      <c r="B123" s="85" t="s">
         <v>208</v>
       </c>
       <c r="C123" s="35" t="s">
@@ -5102,8 +5088,8 @@
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A124" s="106"/>
-      <c r="B124" s="85"/>
+      <c r="A124" s="92"/>
+      <c r="B124" s="86"/>
       <c r="C124" s="13" t="s">
         <v>206</v>
       </c>
@@ -5115,8 +5101,8 @@
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A125" s="106"/>
-      <c r="B125" s="85"/>
+      <c r="A125" s="92"/>
+      <c r="B125" s="86"/>
       <c r="C125" s="13" t="s">
         <v>217</v>
       </c>
@@ -5128,8 +5114,8 @@
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A126" s="106"/>
-      <c r="B126" s="85"/>
+      <c r="A126" s="92"/>
+      <c r="B126" s="86"/>
       <c r="C126" s="13" t="s">
         <v>207</v>
       </c>
@@ -5141,8 +5127,8 @@
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A127" s="106"/>
-      <c r="B127" s="85"/>
+      <c r="A127" s="92"/>
+      <c r="B127" s="86"/>
       <c r="C127" s="13" t="s">
         <v>302</v>
       </c>
@@ -5154,8 +5140,8 @@
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A128" s="106"/>
-      <c r="B128" s="85"/>
+      <c r="A128" s="92"/>
+      <c r="B128" s="86"/>
       <c r="C128" s="44" t="s">
         <v>326</v>
       </c>
@@ -5168,8 +5154,8 @@
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A129" s="106"/>
-      <c r="B129" s="85"/>
+      <c r="A129" s="92"/>
+      <c r="B129" s="86"/>
       <c r="C129" s="44" t="s">
         <v>328</v>
       </c>
@@ -5182,8 +5168,8 @@
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A130" s="106"/>
-      <c r="B130" s="85"/>
+      <c r="A130" s="92"/>
+      <c r="B130" s="86"/>
       <c r="C130" s="13" t="s">
         <v>219</v>
       </c>
@@ -5195,8 +5181,8 @@
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A131" s="106"/>
-      <c r="B131" s="85"/>
+      <c r="A131" s="92"/>
+      <c r="B131" s="86"/>
       <c r="C131" s="13" t="s">
         <v>223</v>
       </c>
@@ -5208,8 +5194,8 @@
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A132" s="106"/>
-      <c r="B132" s="85"/>
+      <c r="A132" s="92"/>
+      <c r="B132" s="86"/>
       <c r="C132" s="13" t="s">
         <v>204</v>
       </c>
@@ -5221,8 +5207,8 @@
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A133" s="106"/>
-      <c r="B133" s="85"/>
+      <c r="A133" s="92"/>
+      <c r="B133" s="86"/>
       <c r="C133" s="44" t="s">
         <v>251</v>
       </c>
@@ -5235,8 +5221,8 @@
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A134" s="106"/>
-      <c r="B134" s="85"/>
+      <c r="A134" s="92"/>
+      <c r="B134" s="86"/>
       <c r="C134" s="44" t="s">
         <v>367</v>
       </c>
@@ -5249,16 +5235,16 @@
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A135" s="106"/>
-      <c r="B135" s="85"/>
+      <c r="A135" s="92"/>
+      <c r="B135" s="86"/>
       <c r="C135" s="44"/>
       <c r="D135" s="44"/>
       <c r="E135" s="44"/>
       <c r="F135" s="44"/>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A136" s="106"/>
-      <c r="B136" s="84" t="s">
+      <c r="A136" s="92"/>
+      <c r="B136" s="85" t="s">
         <v>224</v>
       </c>
       <c r="C136" s="35" t="s">
@@ -5273,8 +5259,8 @@
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A137" s="106"/>
-      <c r="B137" s="102"/>
+      <c r="A137" s="92"/>
+      <c r="B137" s="90"/>
       <c r="C137" s="13" t="s">
         <v>304</v>
       </c>
@@ -5286,8 +5272,8 @@
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A138" s="106"/>
-      <c r="B138" s="102"/>
+      <c r="A138" s="92"/>
+      <c r="B138" s="90"/>
       <c r="C138" s="13" t="s">
         <v>227</v>
       </c>
@@ -5299,8 +5285,8 @@
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A139" s="106"/>
-      <c r="B139" s="102"/>
+      <c r="A139" s="92"/>
+      <c r="B139" s="90"/>
       <c r="C139" s="44" t="s">
         <v>253</v>
       </c>
@@ -5313,8 +5299,8 @@
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A140" s="106"/>
-      <c r="B140" s="102"/>
+      <c r="A140" s="92"/>
+      <c r="B140" s="90"/>
       <c r="C140" s="44" t="s">
         <v>368</v>
       </c>
@@ -5327,12 +5313,12 @@
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A141" s="106"/>
-      <c r="B141" s="102"/>
+      <c r="A141" s="92"/>
+      <c r="B141" s="90"/>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A142" s="106"/>
-      <c r="B142" s="103" t="s">
+      <c r="A142" s="92"/>
+      <c r="B142" s="88" t="s">
         <v>370</v>
       </c>
       <c r="C142" s="35" t="s">
@@ -5347,21 +5333,30 @@
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A143" s="106"/>
-      <c r="B143" s="104"/>
-      <c r="C143" s="105" t="s">
+      <c r="A143" s="92"/>
+      <c r="B143" s="89"/>
+      <c r="C143" s="69" t="s">
         <v>373</v>
       </c>
-      <c r="D143" s="105" t="s">
+      <c r="D143" s="69" t="s">
         <v>374</v>
       </c>
-      <c r="E143" s="105"/>
-      <c r="F143" s="105" t="s">
+      <c r="E143" s="69"/>
+      <c r="F143" s="69" t="s">
         <v>347</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A2:A43"/>
+    <mergeCell ref="B2:B11"/>
+    <mergeCell ref="B12:B22"/>
+    <mergeCell ref="B33:B43"/>
+    <mergeCell ref="A44:A75"/>
+    <mergeCell ref="B64:B75"/>
+    <mergeCell ref="B23:B32"/>
+    <mergeCell ref="B44:B53"/>
+    <mergeCell ref="B54:B63"/>
     <mergeCell ref="B142:B143"/>
     <mergeCell ref="B136:B141"/>
     <mergeCell ref="A113:A143"/>
@@ -5377,15 +5372,6 @@
     <mergeCell ref="B107:B109"/>
     <mergeCell ref="B99:B102"/>
     <mergeCell ref="B103:B106"/>
-    <mergeCell ref="A2:A43"/>
-    <mergeCell ref="B2:B11"/>
-    <mergeCell ref="B12:B22"/>
-    <mergeCell ref="B33:B43"/>
-    <mergeCell ref="A44:A75"/>
-    <mergeCell ref="B64:B75"/>
-    <mergeCell ref="B23:B32"/>
-    <mergeCell ref="B44:B53"/>
-    <mergeCell ref="B54:B63"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>